<commit_message>
2026 Wild Card Results
</commit_message>
<xml_diff>
--- a/2026_results.xlsx
+++ b/2026_results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://newcastle-my.sharepoint.com/personal/nbr37_newcastle_ac_uk/Documents/MEP and Teaching/MMM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="977" documentId="8_{112114C6-7F5F-4BD2-B7B9-FFD9C9F22994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6DE26A63-3810-4039-A6C8-7159697813B9}"/>
+  <xr:revisionPtr revIDLastSave="983" documentId="8_{112114C6-7F5F-4BD2-B7B9-FFD9C9F22994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A8B3B76-42A6-4BF9-AA55-E9F40B0405B0}"/>
   <bookViews>
-    <workbookView xWindow="2880" yWindow="2025" windowWidth="21600" windowHeight="12735" xr2:uid="{3E5A4F85-4087-E24D-A3B4-5C3AA07B2567}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="17640" xr2:uid="{3E5A4F85-4087-E24D-A3B4-5C3AA07B2567}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="78">
   <si>
     <t>Round_1</t>
   </si>
@@ -316,14 +316,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -874,7 +873,6 @@
       </c>
       <c r="G13" s="3"/>
       <c r="M13" s="3"/>
-      <c r="N13" s="4"/>
       <c r="P13" s="3" t="s">
         <v>57</v>
       </c>
@@ -962,7 +960,9 @@
       <c r="A19" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="3"/>
+      <c r="B19" s="3" t="s">
+        <v>30</v>
+      </c>
       <c r="C19">
         <v>1</v>
       </c>
@@ -986,7 +986,9 @@
       <c r="C20">
         <v>16</v>
       </c>
-      <c r="D20" s="3"/>
+      <c r="D20" s="3" t="s">
+        <v>30</v>
+      </c>
       <c r="F20" s="3"/>
       <c r="N20" s="3"/>
       <c r="P20" s="3" t="s">

</xml_diff>

<commit_message>
MMM 2026 money mammals results 1
</commit_message>
<xml_diff>
--- a/2026_results.xlsx
+++ b/2026_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://newcastle-my.sharepoint.com/personal/nbr37_newcastle_ac_uk/Documents/MEP and Teaching/MMM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="983" documentId="8_{112114C6-7F5F-4BD2-B7B9-FFD9C9F22994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A8B3B76-42A6-4BF9-AA55-E9F40B0405B0}"/>
+  <xr:revisionPtr revIDLastSave="991" documentId="8_{112114C6-7F5F-4BD2-B7B9-FFD9C9F22994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E04F3B66-3268-43E3-B8F8-49132EBF54BD}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="17640" xr2:uid="{3E5A4F85-4087-E24D-A3B4-5C3AA07B2567}"/>
+    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{3E5A4F85-4087-E24D-A3B4-5C3AA07B2567}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="78">
   <si>
     <t>Round_1</t>
   </si>
@@ -692,7 +692,9 @@
         <v>9</v>
       </c>
       <c r="E2" s="3"/>
-      <c r="O2" s="3"/>
+      <c r="O2" s="3" t="s">
+        <v>46</v>
+      </c>
       <c r="P2" s="3" t="s">
         <v>46</v>
       </c>
@@ -727,7 +729,9 @@
         <v>15</v>
       </c>
       <c r="E4" s="3"/>
-      <c r="O4" s="3"/>
+      <c r="O4" s="3" t="s">
+        <v>49</v>
+      </c>
       <c r="P4" s="3" t="s">
         <v>48</v>
       </c>
@@ -759,7 +763,9 @@
         <v>17</v>
       </c>
       <c r="E6" s="3"/>
-      <c r="O6" s="3"/>
+      <c r="O6" s="3" t="s">
+        <v>50</v>
+      </c>
       <c r="P6" s="3" t="s">
         <v>50</v>
       </c>
@@ -792,7 +798,9 @@
       </c>
       <c r="E8" s="3"/>
       <c r="H8" s="1"/>
-      <c r="O8" s="3"/>
+      <c r="O8" s="3" t="s">
+        <v>52</v>
+      </c>
       <c r="P8" s="3" t="s">
         <v>52</v>
       </c>
@@ -824,7 +832,9 @@
         <v>21</v>
       </c>
       <c r="E10" s="3"/>
-      <c r="O10" s="3"/>
+      <c r="O10" s="3" t="s">
+        <v>55</v>
+      </c>
       <c r="P10" s="3" t="s">
         <v>54</v>
       </c>
@@ -856,7 +866,9 @@
         <v>23</v>
       </c>
       <c r="E12" s="3"/>
-      <c r="O12" s="3"/>
+      <c r="O12" s="3" t="s">
+        <v>56</v>
+      </c>
       <c r="P12" s="3" t="s">
         <v>56</v>
       </c>
@@ -889,7 +901,9 @@
       </c>
       <c r="E14" s="3"/>
       <c r="M14" s="3"/>
-      <c r="O14" s="3"/>
+      <c r="O14" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="P14" s="3" t="s">
         <v>58</v>
       </c>
@@ -921,7 +935,9 @@
         <v>27</v>
       </c>
       <c r="E16" s="3"/>
-      <c r="O16" s="3"/>
+      <c r="O16" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="P16" s="3" t="s">
         <v>60</v>
       </c>

</xml_diff>

<commit_message>
MMM 2026 Library results 1
</commit_message>
<xml_diff>
--- a/2026_results.xlsx
+++ b/2026_results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://newcastle-my.sharepoint.com/personal/nbr37_newcastle_ac_uk/Documents/MEP and Teaching/MMM/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nbr37\OneDrive - Newcastle University\MEP and Teaching\MMM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="991" documentId="8_{112114C6-7F5F-4BD2-B7B9-FFD9C9F22994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E04F3B66-3268-43E3-B8F8-49132EBF54BD}"/>
+  <xr:revisionPtr revIDLastSave="999" documentId="8_{112114C6-7F5F-4BD2-B7B9-FFD9C9F22994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32729789-5D4C-4323-A414-96F046332E60}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{3E5A4F85-4087-E24D-A3B4-5C3AA07B2567}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{3E5A4F85-4087-E24D-A3B4-5C3AA07B2567}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="78">
   <si>
     <t>Round_1</t>
   </si>
@@ -691,7 +691,9 @@
       <c r="D2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="3"/>
+      <c r="E2" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="O2" s="3" t="s">
         <v>46</v>
       </c>
@@ -728,7 +730,9 @@
       <c r="D4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="3"/>
+      <c r="E4" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="O4" s="3" t="s">
         <v>49</v>
       </c>
@@ -762,7 +766,9 @@
       <c r="D6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="3"/>
+      <c r="E6" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="O6" s="3" t="s">
         <v>50</v>
       </c>
@@ -796,7 +802,9 @@
       <c r="D8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="3"/>
+      <c r="E8" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="H8" s="1"/>
       <c r="O8" s="3" t="s">
         <v>52</v>
@@ -831,7 +839,9 @@
       <c r="D10" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E10" s="3"/>
+      <c r="E10" s="3" t="s">
+        <v>21</v>
+      </c>
       <c r="O10" s="3" t="s">
         <v>55</v>
       </c>
@@ -865,7 +875,9 @@
       <c r="D12" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E12" s="3"/>
+      <c r="E12" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="O12" s="3" t="s">
         <v>56</v>
       </c>
@@ -899,7 +911,9 @@
       <c r="D14" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E14" s="3"/>
+      <c r="E14" s="3" t="s">
+        <v>25</v>
+      </c>
       <c r="M14" s="3"/>
       <c r="O14" s="3" t="s">
         <v>58</v>
@@ -934,7 +948,9 @@
       <c r="D16" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E16" s="3"/>
+      <c r="E16" s="3" t="s">
+        <v>27</v>
+      </c>
       <c r="O16" s="3" t="s">
         <v>60</v>
       </c>

</xml_diff>

<commit_message>
Round 2 2 Results
</commit_message>
<xml_diff>
--- a/2026_results.xlsx
+++ b/2026_results.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nbr37\OneDrive - Newcastle University\MEP and Teaching\MMM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://newcastle-my.sharepoint.com/personal/nbr37_newcastle_ac_uk/Documents/MEP and Teaching/MMM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="999" documentId="8_{112114C6-7F5F-4BD2-B7B9-FFD9C9F22994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32729789-5D4C-4323-A414-96F046332E60}"/>
+  <xr:revisionPtr revIDLastSave="1031" documentId="8_{112114C6-7F5F-4BD2-B7B9-FFD9C9F22994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A047F46-8183-4332-B37C-4EC240E50878}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{3E5A4F85-4087-E24D-A3B4-5C3AA07B2567}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="78">
   <si>
     <t>Round_1</t>
   </si>
@@ -714,8 +714,12 @@
       <c r="D3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="3"/>
-      <c r="N3" s="3"/>
+      <c r="F3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>46</v>
+      </c>
       <c r="P3" s="3" t="s">
         <v>47</v>
       </c>
@@ -786,8 +790,12 @@
       <c r="D7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="3"/>
-      <c r="N7" s="3"/>
+      <c r="F7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>52</v>
+      </c>
       <c r="P7" s="3" t="s">
         <v>51</v>
       </c>
@@ -859,8 +867,12 @@
       <c r="D11" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F11" s="3"/>
-      <c r="N11" s="3"/>
+      <c r="F11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="N11" s="3" t="s">
+        <v>56</v>
+      </c>
       <c r="P11" s="3" t="s">
         <v>55</v>
       </c>
@@ -932,8 +944,12 @@
       <c r="D15" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F15" s="3"/>
-      <c r="N15" s="3"/>
+      <c r="F15" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="N15" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="P15" s="3" t="s">
         <v>59</v>
       </c>
@@ -1001,9 +1017,13 @@
       <c r="D19" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E19" s="3"/>
+      <c r="E19" s="3" t="s">
+        <v>31</v>
+      </c>
       <c r="J19" s="3"/>
-      <c r="O19" s="3"/>
+      <c r="O19" s="3" t="s">
+        <v>62</v>
+      </c>
       <c r="P19" s="3" t="s">
         <v>62</v>
       </c>
@@ -1021,8 +1041,12 @@
       <c r="D20" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F20" s="3"/>
-      <c r="N20" s="3"/>
+      <c r="F20" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N20" s="3" t="s">
+        <v>62</v>
+      </c>
       <c r="P20" s="3" t="s">
         <v>63</v>
       </c>
@@ -1037,8 +1061,12 @@
       <c r="D21" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E21" s="3"/>
-      <c r="O21" s="3"/>
+      <c r="E21" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="O21" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="P21" s="3" t="s">
         <v>64</v>
       </c>
@@ -1069,8 +1097,12 @@
       <c r="D23" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E23" s="3"/>
-      <c r="O23" s="3"/>
+      <c r="E23" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="O23" s="3" t="s">
+        <v>66</v>
+      </c>
       <c r="P23" s="3" t="s">
         <v>66</v>
       </c>
@@ -1085,8 +1117,12 @@
       <c r="D24" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="F24" s="3"/>
-      <c r="N24" s="3"/>
+      <c r="F24" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="N24" s="3" t="s">
+        <v>66</v>
+      </c>
       <c r="P24" s="3" t="s">
         <v>67</v>
       </c>
@@ -1101,8 +1137,12 @@
       <c r="D25" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E25" s="3"/>
-      <c r="O25" s="3"/>
+      <c r="E25" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="O25" s="3" t="s">
+        <v>69</v>
+      </c>
       <c r="P25" s="3" t="s">
         <v>68</v>
       </c>
@@ -1133,8 +1173,12 @@
       <c r="D27" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E27" s="3"/>
-      <c r="O27" s="3"/>
+      <c r="E27" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="O27" s="3" t="s">
+        <v>70</v>
+      </c>
       <c r="P27" s="3" t="s">
         <v>70</v>
       </c>
@@ -1149,8 +1193,12 @@
       <c r="D28" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="F28" s="3"/>
-      <c r="N28" s="3"/>
+      <c r="F28" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="N28" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P28" s="3" t="s">
         <v>71</v>
       </c>
@@ -1165,8 +1213,12 @@
       <c r="D29" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E29" s="3"/>
-      <c r="O29" s="3"/>
+      <c r="E29" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="O29" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="P29" s="3" t="s">
         <v>72</v>
       </c>
@@ -1198,8 +1250,12 @@
       <c r="D31" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E31" s="3"/>
-      <c r="O31" s="3"/>
+      <c r="E31" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="O31" s="3" t="s">
+        <v>75</v>
+      </c>
       <c r="P31" s="3" t="s">
         <v>74</v>
       </c>
@@ -1214,8 +1270,12 @@
       <c r="D32" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="F32" s="3"/>
-      <c r="N32" s="3"/>
+      <c r="F32" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="N32" s="3" t="s">
+        <v>76</v>
+      </c>
       <c r="P32" s="3" t="s">
         <v>75</v>
       </c>
@@ -1230,8 +1290,12 @@
       <c r="D33" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="E33" s="3"/>
-      <c r="O33" s="3"/>
+      <c r="E33" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="O33" s="3" t="s">
+        <v>76</v>
+      </c>
       <c r="P33" s="3" t="s">
         <v>76</v>
       </c>

</xml_diff>